<commit_message>
[Feat] UIDestiny 구현 끝
</commit_message>
<xml_diff>
--- a/Assets/Excel/StageModifierSO.xlsx
+++ b/Assets/Excel/StageModifierSO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whals\OneDrive\Desktop\workspace\TeamProject_CheerUpMyHero\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4885EDA-3B12-4884-A79D-A694BB71077E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2665EA5C-FECC-4811-A5BE-5984610BFD7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4640" yWindow="870" windowWidth="18540" windowHeight="15410" activeTab="2" xr2:uid="{EFCB9097-03F9-4FEA-8889-6DF9B346DC94}"/>
+    <workbookView xWindow="5770" yWindow="3880" windowWidth="18540" windowHeight="15410" activeTab="2" xr2:uid="{EFCB9097-03F9-4FEA-8889-6DF9B346DC94}"/>
   </bookViews>
   <sheets>
     <sheet name="DestinyEffects" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="82">
   <si>
     <t>idNumber</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -320,6 +320,10 @@
   </si>
   <si>
     <t>maxLevel</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>pointPerLevel</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1347,7 +1351,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05532CA7-F06E-4199-AF52-A751CE55BB11}">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9.5" style="1" bestFit="1" customWidth="1"/>
@@ -1355,13 +1359,14 @@
     <col min="3" max="3" width="17.9140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.1640625" customWidth="1"/>
-    <col min="7" max="7" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="32.08203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.75" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="32.08203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1383,11 +1388,14 @@
       <c r="G1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="I1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A2" s="1">
         <v>9030001</v>
       </c>
@@ -1409,8 +1417,11 @@
       <c r="G2">
         <v>-5</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="H2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3" s="1">
         <v>9030002</v>
       </c>
@@ -1432,8 +1443,11 @@
       <c r="G3">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="H3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A4" s="1">
         <v>9030003</v>
       </c>
@@ -1455,8 +1469,11 @@
       <c r="G4">
         <v>-5</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="H4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A5" s="1">
         <v>9030004</v>
       </c>
@@ -1478,8 +1495,11 @@
       <c r="G5">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="H5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" s="1">
         <v>9030005</v>
       </c>
@@ -1501,8 +1521,11 @@
       <c r="G6">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="H6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" s="1">
         <v>9030006</v>
       </c>
@@ -1524,8 +1547,11 @@
       <c r="G7">
         <v>-10</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="H7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <v>9030007</v>
       </c>
@@ -1547,8 +1573,11 @@
       <c r="G8">
         <v>-10</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="H8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
         <v>9030008</v>
       </c>
@@ -1570,8 +1599,11 @@
       <c r="G9">
         <v>10</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="H9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
         <v>9030009</v>
       </c>
@@ -1581,11 +1613,14 @@
       <c r="F10">
         <v>1</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10">
+        <v>4</v>
+      </c>
+      <c r="I10" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A11" s="1">
         <v>9030010</v>
       </c>
@@ -1595,12 +1630,16 @@
       <c r="F11">
         <v>3</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11">
+        <v>4</v>
+      </c>
+      <c r="I11" t="s">
         <v>76</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>